<commit_message>
feat: varredura retroativa ate 11/10 com 52 lojas e 4287 pedidos resgatados mantendo semanas 14 a 20 ate 05 a 11
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-05).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-05).xlsx
@@ -935,22 +935,22 @@
     <t>214</t>
   </si>
   <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>R$ 3.086,12</t>
-  </si>
-  <si>
-    <t>36.2</t>
-  </si>
-  <si>
-    <t>22.0</t>
-  </si>
-  <si>
-    <t>4.55</t>
-  </si>
-  <si>
-    <t>18.7</t>
+    <t>30</t>
+  </si>
+  <si>
+    <t>R$ 3.077,28</t>
+  </si>
+  <si>
+    <t>36.1</t>
+  </si>
+  <si>
+    <t>21.9</t>
+  </si>
+  <si>
+    <t>4.56</t>
+  </si>
+  <si>
+    <t>18.8</t>
   </si>
   <si>
     <t>7.8</t>
@@ -959,10 +959,10 @@
     <t>6.1</t>
   </si>
   <si>
-    <t>45.0%</t>
-  </si>
-  <si>
-    <t>19.3%</t>
+    <t>44.9%</t>
+  </si>
+  <si>
+    <t>19.4%</t>
   </si>
   <si>
     <t>1.6%</t>
@@ -971,7 +971,7 @@
     <t>0.3%</t>
   </si>
   <si>
-    <t>5.2%</t>
+    <t>5.3%</t>
   </si>
   <si>
     <t>1.8%</t>
@@ -983,16 +983,16 @@
     <t>7.7%</t>
   </si>
   <si>
-    <t>3.2%</t>
-  </si>
-  <si>
-    <t>3.8%</t>
-  </si>
-  <si>
-    <t>967.0</t>
-  </si>
-  <si>
-    <t>769.0</t>
+    <t>3.3%</t>
+  </si>
+  <si>
+    <t>3.9%</t>
+  </si>
+  <si>
+    <t>974.0</t>
+  </si>
+  <si>
+    <t>773.0</t>
   </si>
   <si>
     <t>63.0</t>
@@ -1001,22 +1001,22 @@
     <t>11.0</t>
   </si>
   <si>
-    <t>209.0</t>
-  </si>
-  <si>
-    <t>70.0</t>
+    <t>211.0</t>
+  </si>
+  <si>
+    <t>71.0</t>
   </si>
   <si>
     <t>7.0</t>
   </si>
   <si>
-    <t>305.0</t>
-  </si>
-  <si>
-    <t>129.0</t>
-  </si>
-  <si>
-    <t>152.0</t>
+    <t>306.0</t>
+  </si>
+  <si>
+    <t>130.0</t>
+  </si>
+  <si>
+    <t>154.0</t>
   </si>
   <si>
     <t>0.8%</t>
@@ -16689,7 +16689,7 @@
         <v>19719</v>
       </c>
       <c r="B102" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C102" s="4">
         <v>51</v>
@@ -16719,35 +16719,93 @@
         <v>58</v>
       </c>
       <c r="L102" s="4"/>
-      <c r="M102" s="5"/>
-      <c r="N102" s="6"/>
-      <c r="O102" s="6"/>
-      <c r="P102" s="7"/>
-      <c r="Q102" s="8"/>
-      <c r="R102" s="8"/>
-      <c r="S102" s="8"/>
-      <c r="T102" s="9"/>
-      <c r="U102" s="9"/>
-      <c r="V102" s="9"/>
-      <c r="W102" s="9"/>
-      <c r="X102" s="9"/>
-      <c r="Y102" s="9"/>
-      <c r="Z102" s="9"/>
-      <c r="AA102" s="9"/>
-      <c r="AB102" s="9"/>
-      <c r="AC102" s="9"/>
-      <c r="AD102" s="6"/>
-      <c r="AE102" s="6"/>
-      <c r="AF102" s="6"/>
-      <c r="AG102" s="6"/>
-      <c r="AH102" s="6"/>
-      <c r="AI102" s="6"/>
-      <c r="AJ102" s="6"/>
-      <c r="AK102" s="6"/>
-      <c r="AL102" s="6"/>
-      <c r="AM102" s="6"/>
-      <c r="AN102" s="9"/>
-      <c r="AO102" s="6"/>
+      <c r="M102" s="5">
+        <v>1485.5899999999999</v>
+      </c>
+      <c r="N102" s="6">
+        <v>19</v>
+      </c>
+      <c r="O102" s="6">
+        <v>12</v>
+      </c>
+      <c r="P102" s="7">
+        <v>6.3241649999999998</v>
+      </c>
+      <c r="Q102" s="8">
+        <v>23.844441666666668</v>
+      </c>
+      <c r="R102" s="8">
+        <v>11.140909090909091</v>
+      </c>
+      <c r="S102" s="8">
+        <v>7</v>
+      </c>
+      <c r="T102" s="9">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="U102" s="9">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="V102" s="9">
+        <v>0</v>
+      </c>
+      <c r="W102" s="9">
+        <v>0</v>
+      </c>
+      <c r="X102" s="9">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="Y102" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="Z102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="AB102" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="AC102" s="9">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="AD102" s="6">
+        <v>7</v>
+      </c>
+      <c r="AE102" s="6">
+        <v>4</v>
+      </c>
+      <c r="AF102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH102" s="6">
+        <v>2</v>
+      </c>
+      <c r="AI102" s="6">
+        <v>1</v>
+      </c>
+      <c r="AJ102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK102" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL102" s="6">
+        <v>1</v>
+      </c>
+      <c r="AM102" s="6">
+        <v>2</v>
+      </c>
+      <c r="AN102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO102" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP102" s="4">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
feat: varredura e atualizacao com dia 15/10 (quinta) avancando semana para 12 a 15 e 47 lojas resgatadas
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-05).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-05).xlsx
@@ -938,10 +938,10 @@
     <t>215</t>
   </si>
   <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>R$ 3.087,33</t>
+    <t>28</t>
+  </si>
+  <si>
+    <t>R$ 3.093,75</t>
   </si>
   <si>
     <t>36.3</t>
@@ -950,7 +950,7 @@
     <t>22.2</t>
   </si>
   <si>
-    <t>4.59</t>
+    <t>4.60</t>
   </si>
   <si>
     <t>18.7</t>
@@ -962,7 +962,7 @@
     <t>6.2</t>
   </si>
   <si>
-    <t>44.6%</t>
+    <t>44.7%</t>
   </si>
   <si>
     <t>20.2%</t>
@@ -25199,7 +25199,7 @@
         <v>19863</v>
       </c>
       <c r="B159" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C159" s="4">
         <v>51</v>
@@ -25229,18 +25229,30 @@
         <v>58</v>
       </c>
       <c r="L159" s="4"/>
-      <c r="M159" s="5"/>
-      <c r="N159" s="6"/>
+      <c r="M159" s="5">
+        <v>4266.8699999999999</v>
+      </c>
+      <c r="N159" s="6">
+        <v>47</v>
+      </c>
       <c r="O159" s="6">
         <v>32</v>
       </c>
-      <c r="P159" s="7"/>
-      <c r="Q159" s="8"/>
-      <c r="R159" s="8"/>
+      <c r="P159" s="7">
+        <v>6.1739130434782608</v>
+      </c>
+      <c r="Q159" s="8">
+        <v>19.618749999999999</v>
+      </c>
+      <c r="R159" s="8">
+        <v>6.4144433333333337</v>
+      </c>
       <c r="S159" s="8">
         <v>7</v>
       </c>
-      <c r="T159" s="9"/>
+      <c r="T159" s="9">
+        <v>0.1875</v>
+      </c>
       <c r="U159" s="9">
         <v>0.09375</v>
       </c>

</xml_diff>